<commit_message>
Employee Excel sheet Import IP number include
</commit_message>
<xml_diff>
--- a/assets/download/ActiveMember_NEW.xlsx
+++ b/assets/download/ActiveMember_NEW.xlsx
@@ -1,22 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId5"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+  <si>
+    <t>Uan</t>
+  </si>
+  <si>
+    <t>IP Number</t>
+  </si>
+  <si>
+    <t>MemberId</t>
+  </si>
+  <si>
+    <t>Ccode</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
   <si>
     <t>Name</t>
   </si>
@@ -54,6 +70,18 @@
     <t>Bank</t>
   </si>
   <si>
+    <t>Nationatily</t>
+  </si>
+  <si>
+    <t>PMRPY</t>
+  </si>
+  <si>
+    <t>IFSC CODE</t>
+  </si>
+  <si>
+    <t>WBDGP00340830000000036</t>
+  </si>
+  <si>
     <t>BIDI PACKER</t>
   </si>
   <si>
@@ -75,77 +103,64 @@
     <t>INDIAN</t>
   </si>
   <si>
-    <t>Uan</t>
-  </si>
-  <si>
-    <t>MemberId</t>
-  </si>
-  <si>
-    <t>WBDGP00340830000000036</t>
-  </si>
-  <si>
-    <t>Ccode</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>Nationatily</t>
-  </si>
-  <si>
-    <t>PMRPY</t>
-  </si>
-  <si>
     <t>YES</t>
-  </si>
-  <si>
-    <t>IFSC CODE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="15" fillId="2" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="1" fillId="2" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -224,6 +239,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -258,6 +274,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -433,160 +450,205 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="31.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" customWidth="1"/>
-    <col min="9" max="9" width="21.5703125" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" customWidth="1"/>
-    <col min="11" max="11" width="17.5703125" customWidth="1"/>
-    <col min="12" max="12" width="11" customWidth="1"/>
-    <col min="13" max="13" width="31.7109375" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" customWidth="1"/>
-    <col min="15" max="15" width="15.5703125" customWidth="1"/>
-    <col min="16" max="16" width="14.28515625" customWidth="1"/>
-    <col min="17" max="17" width="12.140625" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="true" style="0"/>
+    <col min="3" max="3" width="24.7109375" customWidth="true" style="0"/>
+    <col min="4" max="4" width="16.140625" customWidth="true" style="0"/>
+    <col min="5" max="5" width="15.85546875" customWidth="true" style="0"/>
+    <col min="6" max="6" width="31.7109375" customWidth="true" style="0"/>
+    <col min="7" max="7" width="12.28515625" customWidth="true" style="0"/>
+    <col min="9" max="9" width="11.28515625" customWidth="true" style="0"/>
+    <col min="10" max="10" width="21.5703125" customWidth="true" style="0"/>
+    <col min="11" max="11" width="13.85546875" customWidth="true" style="0"/>
+    <col min="12" max="12" width="17.5703125" customWidth="true" style="0"/>
+    <col min="13" max="13" width="11" customWidth="true" style="0"/>
+    <col min="14" max="14" width="31.7109375" customWidth="true" style="0"/>
+    <col min="15" max="15" width="13.5703125" customWidth="true" style="0"/>
+    <col min="16" max="16" width="15.5703125" customWidth="true" style="0"/>
+    <col min="17" max="17" width="14.28515625" customWidth="true" style="0"/>
+    <col min="18" max="18" width="12.140625" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:20">
       <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" t="s">
-        <v>8</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" t="s">
-        <v>10</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>24</v>
-      </c>
-      <c r="R1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S1" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:20">
       <c r="A2" s="2">
         <v>100364405278</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="1">
+      <c r="F2" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="1">
         <v>28511</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="1">
         <v>35886</v>
       </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" t="s">
-        <v>17</v>
-      </c>
-      <c r="L2">
+      <c r="J2" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" s="0">
         <v>9775348353</v>
       </c>
-      <c r="M2" s="3" t="str">
-        <f>N2&amp;"@DINESHBIDI.COM"</f>
-        <v>847738128184@DINESHBIDI.COM</v>
-      </c>
-      <c r="N2" s="2">
+      <c r="N2" s="3" t="str">
+        <f>O2&amp;"@DINESHBIDI.COM"</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="2">
         <v>847738128184</v>
       </c>
-      <c r="O2" t="s">
-        <v>17</v>
-      </c>
-      <c r="P2" s="2">
+      <c r="P2" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q2" s="2">
         <v>1334010212038</v>
       </c>
-      <c r="Q2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R2" t="s">
-        <v>26</v>
+      <c r="R2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2" s="0" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
+  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
+  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
employee bulk and uan to ip mapping excel format
</commit_message>
<xml_diff>
--- a/assets/download/ActiveMember_NEW.xlsx
+++ b/assets/download/ActiveMember_NEW.xlsx
@@ -7,9 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId5"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId6"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
@@ -17,93 +15,105 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
-  <si>
-    <t>Uan</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="33">
+  <si>
+    <t>Note: Columns marked with * are mandatory to fill.</t>
+  </si>
+  <si>
+    <t>UAN*</t>
   </si>
   <si>
     <t>IP Number</t>
   </si>
   <si>
-    <t>MemberId</t>
-  </si>
-  <si>
-    <t>Ccode</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>Name</t>
+    <t>Previous Member ID</t>
+  </si>
+  <si>
+    <t>Contractor Code</t>
+  </si>
+  <si>
+    <t>Employee Type</t>
+  </si>
+  <si>
+    <t>Employee Name</t>
   </si>
   <si>
     <t>Gender</t>
   </si>
   <si>
-    <t>Dob</t>
-  </si>
-  <si>
-    <t>Doj</t>
-  </si>
-  <si>
-    <t>FatherOrHusbandName</t>
+    <t>DOB (DD-MM-YYYY)</t>
+  </si>
+  <si>
+    <t>DOJ (DD-MM-YYYY)</t>
+  </si>
+  <si>
+    <t>Father/Husband Name</t>
   </si>
   <si>
     <t>Relation</t>
   </si>
   <si>
-    <t>MaritalStatus</t>
+    <t>Marital Status</t>
   </si>
   <si>
     <t>Mobile</t>
   </si>
   <si>
-    <t>EmailId</t>
-  </si>
-  <si>
-    <t>Aadhar</t>
-  </si>
-  <si>
-    <t>Pan</t>
-  </si>
-  <si>
-    <t>Bank</t>
-  </si>
-  <si>
-    <t>Nationatily</t>
+    <t>Aadhaar No</t>
+  </si>
+  <si>
+    <t>PAN</t>
+  </si>
+  <si>
+    <t>Bank Acc No</t>
+  </si>
+  <si>
+    <t>Nationality</t>
   </si>
   <si>
     <t>PMRPY</t>
   </si>
   <si>
-    <t>IFSC CODE</t>
-  </si>
-  <si>
-    <t>WBDGP00340830000000036</t>
-  </si>
-  <si>
-    <t>BIDI PACKER</t>
-  </si>
-  <si>
-    <t>Mr. SUBHENDU KUMAR</t>
+    <t>IFSC</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>OFFICE STAFF</t>
+  </si>
+  <si>
+    <t>JOHN DOE</t>
   </si>
   <si>
     <t>MALE</t>
   </si>
   <si>
-    <t>ARJUN KUMAR</t>
+    <t>01-01-1990</t>
+  </si>
+  <si>
+    <t>01-01-2020</t>
+  </si>
+  <si>
+    <t>RICHARD DOE</t>
   </si>
   <si>
     <t>FATHER</t>
   </si>
   <si>
-    <t>NOT AVAILABLE</t>
+    <t>MARRIED</t>
+  </si>
+  <si>
+    <t>ABCDE1234F</t>
   </si>
   <si>
     <t>INDIAN</t>
   </si>
   <si>
     <t>YES</t>
+  </si>
+  <si>
+    <t>SBIN0001234</t>
   </si>
 </sst>
 </file>
@@ -111,7 +121,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -121,8 +131,17 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -132,9 +151,6 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -142,17 +158,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
+  <cellXfs count="2">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="15" fillId="2" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="1" fillId="2" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
@@ -454,141 +464,151 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="true" style="0"/>
-    <col min="3" max="3" width="24.7109375" customWidth="true" style="0"/>
-    <col min="4" max="4" width="16.140625" customWidth="true" style="0"/>
-    <col min="5" max="5" width="15.85546875" customWidth="true" style="0"/>
-    <col min="6" max="6" width="31.7109375" customWidth="true" style="0"/>
-    <col min="7" max="7" width="12.28515625" customWidth="true" style="0"/>
-    <col min="9" max="9" width="11.28515625" customWidth="true" style="0"/>
-    <col min="10" max="10" width="21.5703125" customWidth="true" style="0"/>
-    <col min="11" max="11" width="13.85546875" customWidth="true" style="0"/>
-    <col min="12" max="12" width="17.5703125" customWidth="true" style="0"/>
-    <col min="13" max="13" width="11" customWidth="true" style="0"/>
-    <col min="14" max="14" width="31.7109375" customWidth="true" style="0"/>
-    <col min="15" max="15" width="13.5703125" customWidth="true" style="0"/>
-    <col min="16" max="16" width="15.5703125" customWidth="true" style="0"/>
-    <col min="17" max="17" width="14.28515625" customWidth="true" style="0"/>
-    <col min="18" max="18" width="12.140625" customWidth="true" style="0"/>
+    <col min="1" max="1" width="60.128174" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="12.854004" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="22.280273" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="18.709717" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="16.424561" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="16.424561" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="8.140869" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="19.995117" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="19.995117" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="23.422852" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="10.568848" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="17.567139" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="12.854004" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="15.281982" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="12.854004" bestFit="true" customWidth="true" style="0"/>
+    <col min="16" max="16" width="13.996582" bestFit="true" customWidth="true" style="0"/>
+    <col min="17" max="17" width="13.996582" bestFit="true" customWidth="true" style="0"/>
+    <col min="18" max="18" width="6.998291" bestFit="true" customWidth="true" style="0"/>
+    <col min="19" max="19" width="13.996582" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:19">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+    </row>
+    <row r="2" spans="1:19">
+      <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="B2" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="C2" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="D2" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="E2" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="F2" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="G2" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="H2" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="I2" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="J2" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="K2" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="L2" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="M2" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="N2" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="0" t="s">
+      <c r="O2" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="P2" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="0" t="s">
+      <c r="Q2" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="0" t="s">
+      <c r="R2" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="0" t="s">
+      <c r="S2" s="0" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
-      <c r="A2" s="2">
-        <v>100364405278</v>
-      </c>
-      <c r="C2" s="0" t="s">
+    <row r="3" spans="1:19">
+      <c r="A3" s="0">
+        <v>123456789012</v>
+      </c>
+      <c r="B3" s="0">
+        <v>1234567890</v>
+      </c>
+      <c r="C3" s="0">
+        <v>10001</v>
+      </c>
+      <c r="D3" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E3" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F3" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G3" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="1">
-        <v>28511</v>
-      </c>
-      <c r="I2" s="1">
-        <v>35886</v>
-      </c>
-      <c r="J2" s="0" t="s">
+      <c r="H3" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="I3" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="J3" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="0">
-        <v>9775348353</v>
-      </c>
-      <c r="N2" s="3" t="str">
-        <f>O2&amp;"@DINESHBIDI.COM"</f>
-        <v>0</v>
-      </c>
-      <c r="O2" s="2">
-        <v>847738128184</v>
-      </c>
-      <c r="P2" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q2" s="2">
-        <v>1334010212038</v>
-      </c>
-      <c r="R2" s="2" t="s">
+      <c r="K3" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="S2" s="0" t="s">
+      <c r="L3" s="0" t="s">
         <v>28</v>
+      </c>
+      <c r="M3" s="0">
+        <v>9876543210</v>
+      </c>
+      <c r="N3" s="0">
+        <v>123412341234</v>
+      </c>
+      <c r="O3" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="P3" s="0">
+        <v>1234567890</v>
+      </c>
+      <c r="Q3" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="R3" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="S3" s="0" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -605,50 +625,4 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
-  <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
-  <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>